<commit_message>
fix: restaurar Remision E0093 (PLANTA RIO XIX, tarimas TPM-0309, TPM-0311, TPM-0317) y actualizar estatus e historial de actividad
</commit_message>
<xml_diff>
--- a/BD_Actividad_Log.xlsx
+++ b/BD_Actividad_Log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J494"/>
+  <dimension ref="A1:J498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22160,6 +22160,198 @@
         </is>
       </c>
     </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>494</v>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>09:35:18</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Remisión E0093 generada con 3 tarima(s) (TPM-0309, TPM-0311, TPM-0317) y 72 piezas hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>E0093</t>
+        </is>
+      </c>
+      <c r="H495" t="n">
+        <v>72</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>495</v>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>09:35:18</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0309 marcada como Remesada en E0093 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>TPM-0309</t>
+        </is>
+      </c>
+      <c r="H496" t="n">
+        <v>24</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>496</v>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>09:35:18</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0311 marcada como Remesada en E0093 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>TPM-0311</t>
+        </is>
+      </c>
+      <c r="H497" t="n">
+        <v>24</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>497</v>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>09:35:18</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0317 marcada como Remesada en E0093 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>TPM-0317</t>
+        </is>
+      </c>
+      <c r="H498" t="n">
+        <v>24</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>